<commit_message>
Finalized 1st shift DSI ppw
</commit_message>
<xml_diff>
--- a/CustomLabelPrinter/src/paperwork/dsi/recap-1st.xlsx
+++ b/CustomLabelPrinter/src/paperwork/dsi/recap-1st.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tdphu\git\customlabelprinter\CustomLabelPrinter\src\paperwork\dsi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\git\CustomLabelPrinter\CustomLabelPrinter\src\paperwork\dsi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C656224-DBF8-434B-A3DB-C0365F6D162C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD88EC83-5D8F-4D0E-8540-1239178ABECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6555" yWindow="810" windowWidth="25665" windowHeight="15960" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="930" yWindow="2010" windowWidth="21600" windowHeight="11295" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Breast" sheetId="2" r:id="rId1"/>
@@ -25,6 +25,9 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -510,15 +513,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -528,9 +528,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -580,6 +577,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -598,15 +599,39 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -903,19 +928,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
     </row>
     <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -930,222 +955,222 @@
     </row>
     <row r="4" spans="1:11" ht="8.4499999999999993" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" s="2" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="30">
+      <c r="B5" s="24">
         <v>8</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="24">
         <v>9</v>
       </c>
-      <c r="D5" s="30">
+      <c r="D5" s="24">
         <v>10</v>
       </c>
-      <c r="E5" s="30">
+      <c r="E5" s="24">
         <v>11</v>
       </c>
-      <c r="F5" s="30">
+      <c r="F5" s="24">
         <v>12</v>
       </c>
-      <c r="G5" s="30">
+      <c r="G5" s="24">
         <v>13</v>
       </c>
-      <c r="H5" s="30">
+      <c r="H5" s="24">
         <v>14</v>
       </c>
-      <c r="I5" s="30">
+      <c r="I5" s="24">
         <v>15</v>
       </c>
-      <c r="J5" s="30">
+      <c r="J5" s="24">
         <v>16</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="K5" s="5" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="32"/>
+      <c r="A6" s="26"/>
     </row>
     <row r="7" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="32"/>
+      <c r="A7" s="26"/>
     </row>
     <row r="8" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="32"/>
+      <c r="A8" s="26"/>
     </row>
     <row r="9" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="32"/>
+      <c r="A9" s="26"/>
     </row>
     <row r="10" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="32"/>
+      <c r="A10" s="26"/>
     </row>
     <row r="11" spans="1:11" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="32"/>
+      <c r="A11" s="26"/>
     </row>
     <row r="12" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="32"/>
+      <c r="A12" s="26"/>
     </row>
     <row r="13" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="32"/>
+      <c r="A13" s="26"/>
     </row>
     <row r="14" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="32"/>
+      <c r="A14" s="26"/>
     </row>
     <row r="15" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="32"/>
+      <c r="A15" s="26"/>
     </row>
     <row r="16" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="32"/>
+      <c r="A16" s="26"/>
     </row>
     <row r="17" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="32"/>
+      <c r="A17" s="26"/>
     </row>
     <row r="18" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="32"/>
+      <c r="A18" s="26"/>
     </row>
     <row r="19" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="32"/>
+      <c r="A19" s="26"/>
     </row>
     <row r="20" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="32"/>
+      <c r="A20" s="26"/>
     </row>
     <row r="21" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="32"/>
+      <c r="A21" s="26"/>
     </row>
     <row r="22" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="32"/>
+      <c r="A22" s="26"/>
     </row>
     <row r="23" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="32"/>
+      <c r="A23" s="26"/>
     </row>
     <row r="24" spans="1:1" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="32"/>
+      <c r="A24" s="26"/>
     </row>
     <row r="25" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="32"/>
+      <c r="A25" s="26"/>
     </row>
     <row r="26" spans="1:1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="32"/>
+      <c r="A26" s="26"/>
     </row>
     <row r="27" spans="1:1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="32"/>
+      <c r="A27" s="26"/>
     </row>
     <row r="28" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="32"/>
+      <c r="A28" s="26"/>
     </row>
     <row r="29" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="32"/>
+      <c r="A29" s="26"/>
     </row>
     <row r="30" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="32"/>
+      <c r="A30" s="26"/>
     </row>
     <row r="31" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="32"/>
+      <c r="A31" s="26"/>
     </row>
     <row r="32" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="32"/>
+      <c r="A32" s="26"/>
     </row>
     <row r="33" spans="1:1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="32"/>
+      <c r="A33" s="26"/>
     </row>
     <row r="34" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="32"/>
+      <c r="A34" s="26"/>
     </row>
     <row r="35" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="32"/>
+      <c r="A35" s="26"/>
     </row>
     <row r="36" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="32"/>
+      <c r="A36" s="26"/>
     </row>
     <row r="37" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="32"/>
+      <c r="A37" s="26"/>
     </row>
     <row r="38" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="32"/>
+      <c r="A38" s="26"/>
     </row>
     <row r="39" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="32"/>
+      <c r="A39" s="26"/>
     </row>
     <row r="40" spans="1:1" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="32"/>
+      <c r="A40" s="26"/>
     </row>
     <row r="41" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="32"/>
+      <c r="A41" s="26"/>
     </row>
     <row r="42" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="32"/>
+      <c r="A42" s="26"/>
     </row>
     <row r="43" spans="1:1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="32"/>
+      <c r="A43" s="26"/>
     </row>
     <row r="44" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="32"/>
+      <c r="A44" s="26"/>
     </row>
     <row r="45" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="32"/>
+      <c r="A45" s="26"/>
     </row>
     <row r="46" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="32"/>
+      <c r="A46" s="26"/>
     </row>
     <row r="47" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="32"/>
+      <c r="A47" s="26"/>
     </row>
     <row r="48" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="32"/>
+      <c r="A48" s="26"/>
     </row>
     <row r="49" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="32"/>
+      <c r="A49" s="26"/>
     </row>
     <row r="50" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="32"/>
+      <c r="A50" s="26"/>
     </row>
     <row r="51" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="32"/>
+      <c r="A51" s="26"/>
     </row>
     <row r="52" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="32"/>
+      <c r="A52" s="26"/>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A53" s="10"/>
+      <c r="A53" s="7"/>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54" s="10"/>
+      <c r="A54" s="7"/>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" s="10"/>
+      <c r="A55" s="7"/>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A56" s="10"/>
+      <c r="A56" s="7"/>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A57" s="10"/>
+      <c r="A57" s="7"/>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A58" s="10"/>
+      <c r="A58" s="7"/>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" s="10"/>
+      <c r="A59" s="7"/>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60" s="10"/>
+      <c r="A60" s="7"/>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" s="10"/>
+      <c r="A61" s="7"/>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" s="10"/>
+      <c r="A62" s="7"/>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" s="10"/>
+      <c r="A63" s="7"/>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64" s="10"/>
+      <c r="A64" s="7"/>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A65" s="10"/>
+      <c r="A65" s="7"/>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" s="10"/>
+      <c r="A66" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1174,19 +1199,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="36" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
     </row>
     <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -1201,189 +1226,189 @@
     </row>
     <row r="4" spans="1:11" ht="21.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:11" s="2" customFormat="1" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="30">
+      <c r="B5" s="24">
         <v>8</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="24">
         <v>9</v>
       </c>
-      <c r="D5" s="30">
+      <c r="D5" s="24">
         <v>10</v>
       </c>
-      <c r="E5" s="30">
+      <c r="E5" s="24">
         <v>11</v>
       </c>
-      <c r="F5" s="30">
+      <c r="F5" s="24">
         <v>12</v>
       </c>
-      <c r="G5" s="30">
+      <c r="G5" s="24">
         <v>13</v>
       </c>
-      <c r="H5" s="30">
+      <c r="H5" s="24">
         <v>14</v>
       </c>
-      <c r="I5" s="30">
+      <c r="I5" s="24">
         <v>15</v>
       </c>
-      <c r="J5" s="30">
+      <c r="J5" s="24">
         <v>16</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="K5" s="5" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="32"/>
+      <c r="A6" s="26"/>
     </row>
     <row r="7" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="32"/>
+      <c r="A7" s="26"/>
     </row>
     <row r="8" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="32"/>
+      <c r="A8" s="26"/>
     </row>
     <row r="9" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="32"/>
+      <c r="A9" s="26"/>
     </row>
     <row r="10" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="32"/>
+      <c r="A10" s="26"/>
     </row>
     <row r="11" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="32"/>
+      <c r="A11" s="26"/>
     </row>
     <row r="12" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="32"/>
+      <c r="A12" s="26"/>
     </row>
     <row r="13" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="32"/>
+      <c r="A13" s="26"/>
     </row>
     <row r="14" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="32"/>
+      <c r="A14" s="26"/>
     </row>
     <row r="15" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="32"/>
+      <c r="A15" s="26"/>
     </row>
     <row r="16" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="32"/>
+      <c r="A16" s="26"/>
     </row>
     <row r="17" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="32"/>
+      <c r="A17" s="26"/>
     </row>
     <row r="18" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="32"/>
+      <c r="A18" s="26"/>
     </row>
     <row r="19" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="32"/>
+      <c r="A19" s="26"/>
     </row>
     <row r="20" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="32"/>
+      <c r="A20" s="26"/>
     </row>
     <row r="21" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="32"/>
+      <c r="A21" s="26"/>
     </row>
     <row r="22" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="32"/>
+      <c r="A22" s="26"/>
     </row>
     <row r="23" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="32"/>
+      <c r="A23" s="26"/>
     </row>
     <row r="24" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="32"/>
+      <c r="A24" s="26"/>
     </row>
     <row r="25" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="32"/>
+      <c r="A25" s="26"/>
     </row>
     <row r="26" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="32"/>
+      <c r="A26" s="26"/>
     </row>
     <row r="27" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="32"/>
+      <c r="A27" s="26"/>
     </row>
     <row r="28" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="32"/>
+      <c r="A28" s="26"/>
     </row>
     <row r="29" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="32"/>
+      <c r="A29" s="26"/>
     </row>
     <row r="30" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="32"/>
+      <c r="A30" s="26"/>
     </row>
     <row r="31" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="32"/>
+      <c r="A31" s="26"/>
     </row>
     <row r="32" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="32"/>
+      <c r="A32" s="26"/>
     </row>
     <row r="33" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="32"/>
+      <c r="A33" s="26"/>
     </row>
     <row r="34" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="32"/>
+      <c r="A34" s="26"/>
     </row>
     <row r="35" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="32"/>
+      <c r="A35" s="26"/>
     </row>
     <row r="36" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="32"/>
+      <c r="A36" s="26"/>
     </row>
     <row r="37" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="32"/>
+      <c r="A37" s="26"/>
     </row>
     <row r="38" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="32"/>
+      <c r="A38" s="26"/>
     </row>
     <row r="39" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="32"/>
+      <c r="A39" s="26"/>
     </row>
     <row r="40" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="32"/>
+      <c r="A40" s="26"/>
     </row>
     <row r="41" spans="1:1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="32"/>
+      <c r="A41" s="26"/>
     </row>
     <row r="42" spans="1:1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="32"/>
+      <c r="A42" s="26"/>
     </row>
     <row r="43" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="10"/>
+      <c r="A43" s="7"/>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" s="10"/>
+      <c r="A44" s="7"/>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" s="10"/>
+      <c r="A45" s="7"/>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" s="10"/>
+      <c r="A46" s="7"/>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" s="10"/>
+      <c r="A47" s="7"/>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" s="10"/>
+      <c r="A48" s="7"/>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" s="10"/>
+      <c r="A49" s="7"/>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" s="10"/>
+      <c r="A50" s="7"/>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A51" s="10"/>
+      <c r="A51" s="7"/>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A52" s="10"/>
+      <c r="A52" s="7"/>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A53" s="10"/>
+      <c r="A53" s="7"/>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54" s="10"/>
+      <c r="A54" s="7"/>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" s="10"/>
+      <c r="A55" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1413,443 +1438,443 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
     </row>
     <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
       <c r="I3" s="4"/>
     </row>
     <row r="4" spans="1:11" ht="22.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:11" s="18" customFormat="1" ht="33.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
+    <row r="5" spans="1:11" s="12" customFormat="1" ht="33.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="23">
+      <c r="B5" s="17">
         <v>8</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="13">
         <v>9</v>
       </c>
-      <c r="D5" s="19">
+      <c r="D5" s="13">
         <v>10</v>
       </c>
-      <c r="E5" s="19">
+      <c r="E5" s="13">
         <v>11</v>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="13">
         <v>12</v>
       </c>
-      <c r="G5" s="19">
+      <c r="G5" s="13">
         <v>13</v>
       </c>
-      <c r="H5" s="19">
+      <c r="H5" s="13">
         <v>14</v>
       </c>
-      <c r="I5" s="19">
+      <c r="I5" s="13">
         <v>15</v>
       </c>
-      <c r="J5" s="19">
+      <c r="J5" s="13">
         <v>16</v>
       </c>
-      <c r="K5" s="20" t="s">
+      <c r="K5" s="14" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24">
+      <c r="A6" s="18">
         <v>1</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="43"/>
+      <c r="B6" s="38"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="38"/>
+      <c r="H6" s="38"/>
+      <c r="I6" s="38"/>
+      <c r="J6" s="38"/>
+      <c r="K6" s="44"/>
     </row>
     <row r="7" spans="1:11" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="25">
+      <c r="A7" s="19">
         <v>2</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="7"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="36"/>
+      <c r="K7" s="42"/>
     </row>
     <row r="8" spans="1:11" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25">
+      <c r="A8" s="19">
         <v>3</v>
       </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="7"/>
+      <c r="B8" s="36"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="36"/>
+      <c r="I8" s="36"/>
+      <c r="J8" s="36"/>
+      <c r="K8" s="42"/>
     </row>
     <row r="9" spans="1:11" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="25">
+      <c r="A9" s="19">
         <v>4</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="7"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="36"/>
+      <c r="J9" s="36"/>
+      <c r="K9" s="42"/>
     </row>
     <row r="10" spans="1:11" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="25">
+      <c r="A10" s="19">
         <v>5</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="7"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="36"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="36"/>
+      <c r="H10" s="36"/>
+      <c r="I10" s="36"/>
+      <c r="J10" s="36"/>
+      <c r="K10" s="42"/>
     </row>
     <row r="11" spans="1:11" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="25">
+      <c r="A11" s="19">
         <v>6</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="7"/>
+      <c r="B11" s="36"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="36"/>
+      <c r="E11" s="36"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="36"/>
+      <c r="H11" s="36"/>
+      <c r="I11" s="36"/>
+      <c r="J11" s="36"/>
+      <c r="K11" s="42"/>
     </row>
     <row r="12" spans="1:11" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="25">
+      <c r="A12" s="19">
         <v>7</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="7"/>
+      <c r="B12" s="36"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="36"/>
+      <c r="H12" s="36"/>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36"/>
+      <c r="K12" s="42"/>
     </row>
     <row r="13" spans="1:11" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="25">
+      <c r="A13" s="19">
         <v>8</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="7"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="36"/>
+      <c r="I13" s="36"/>
+      <c r="J13" s="36"/>
+      <c r="K13" s="42"/>
     </row>
     <row r="14" spans="1:11" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="25">
+      <c r="A14" s="19">
         <v>9</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="7"/>
+      <c r="B14" s="36"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="36"/>
+      <c r="I14" s="36"/>
+      <c r="J14" s="36"/>
+      <c r="K14" s="42"/>
     </row>
     <row r="15" spans="1:11" ht="25.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="26">
+      <c r="A15" s="20">
         <v>10</v>
       </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="12"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="37"/>
+      <c r="I15" s="37"/>
+      <c r="J15" s="37"/>
+      <c r="K15" s="43"/>
     </row>
     <row r="16" spans="1:11" ht="25.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="14"/>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="16"/>
-    </row>
-    <row r="17" spans="1:12" s="21" customFormat="1" ht="33.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="17">
+      <c r="A16" s="8"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="10"/>
+    </row>
+    <row r="17" spans="1:12" s="15" customFormat="1" ht="33.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="11">
         <v>21102</v>
       </c>
-      <c r="B17" s="19">
+      <c r="B17" s="13">
         <v>8</v>
       </c>
-      <c r="C17" s="19">
+      <c r="C17" s="13">
         <v>9</v>
       </c>
-      <c r="D17" s="19">
+      <c r="D17" s="13">
         <v>10</v>
       </c>
-      <c r="E17" s="19">
+      <c r="E17" s="13">
         <v>11</v>
       </c>
-      <c r="F17" s="19">
+      <c r="F17" s="13">
         <v>12</v>
       </c>
-      <c r="G17" s="19">
+      <c r="G17" s="13">
         <v>13</v>
       </c>
-      <c r="H17" s="19">
+      <c r="H17" s="13">
         <v>14</v>
       </c>
-      <c r="I17" s="19">
+      <c r="I17" s="13">
         <v>15</v>
       </c>
-      <c r="J17" s="19">
+      <c r="J17" s="13">
         <v>16</v>
       </c>
-      <c r="K17" s="20" t="s">
+      <c r="K17" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="L17" s="31"/>
+      <c r="L17" s="25"/>
     </row>
     <row r="18" spans="1:12" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="27">
+      <c r="A18" s="21">
         <v>1</v>
       </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
-      <c r="K18" s="42"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="35"/>
+      <c r="F18" s="35"/>
+      <c r="G18" s="35"/>
+      <c r="H18" s="35"/>
+      <c r="I18" s="35"/>
+      <c r="J18" s="35"/>
+      <c r="K18" s="41"/>
     </row>
     <row r="19" spans="1:12" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="25">
+      <c r="A19" s="19">
         <v>2</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="7"/>
+      <c r="B19" s="36"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="36"/>
+      <c r="I19" s="36"/>
+      <c r="J19" s="36"/>
+      <c r="K19" s="42"/>
     </row>
     <row r="20" spans="1:12" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="25">
+      <c r="A20" s="19">
         <v>3</v>
       </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="6"/>
-      <c r="J20" s="6"/>
-      <c r="K20" s="7"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="36"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="36"/>
+      <c r="I20" s="36"/>
+      <c r="J20" s="36"/>
+      <c r="K20" s="42"/>
     </row>
     <row r="21" spans="1:12" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="25">
+      <c r="A21" s="19">
         <v>4</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="7"/>
+      <c r="B21" s="36"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="36"/>
+      <c r="F21" s="36"/>
+      <c r="G21" s="36"/>
+      <c r="H21" s="36"/>
+      <c r="I21" s="36"/>
+      <c r="J21" s="36"/>
+      <c r="K21" s="42"/>
     </row>
     <row r="22" spans="1:12" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="25">
+      <c r="A22" s="19">
         <v>5</v>
       </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="7"/>
+      <c r="B22" s="36"/>
+      <c r="C22" s="36"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="36"/>
+      <c r="J22" s="36"/>
+      <c r="K22" s="42"/>
     </row>
     <row r="23" spans="1:12" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="25">
+      <c r="A23" s="19">
         <v>6</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
-      <c r="K23" s="7"/>
+      <c r="B23" s="36"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="36"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="36"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="36"/>
+      <c r="J23" s="36"/>
+      <c r="K23" s="42"/>
     </row>
     <row r="24" spans="1:12" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="25">
+      <c r="A24" s="19">
         <v>7</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
-      <c r="K24" s="7"/>
+      <c r="B24" s="36"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="36"/>
+      <c r="I24" s="36"/>
+      <c r="J24" s="36"/>
+      <c r="K24" s="42"/>
     </row>
     <row r="25" spans="1:12" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="25">
+      <c r="A25" s="19">
         <v>8</v>
       </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
-      <c r="K25" s="7"/>
+      <c r="B25" s="36"/>
+      <c r="C25" s="36"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="36"/>
+      <c r="F25" s="36"/>
+      <c r="G25" s="36"/>
+      <c r="H25" s="36"/>
+      <c r="I25" s="36"/>
+      <c r="J25" s="36"/>
+      <c r="K25" s="42"/>
     </row>
     <row r="26" spans="1:12" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="25">
+      <c r="A26" s="19">
         <v>9</v>
       </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="6"/>
-      <c r="K26" s="7"/>
+      <c r="B26" s="36"/>
+      <c r="C26" s="36"/>
+      <c r="D26" s="36"/>
+      <c r="E26" s="36"/>
+      <c r="F26" s="36"/>
+      <c r="G26" s="36"/>
+      <c r="H26" s="36"/>
+      <c r="I26" s="36"/>
+      <c r="J26" s="36"/>
+      <c r="K26" s="42"/>
     </row>
     <row r="27" spans="1:12" ht="25.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="26">
+      <c r="A27" s="20">
         <v>10</v>
       </c>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="11"/>
-      <c r="K27" s="12"/>
+      <c r="B27" s="37"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="37"/>
+      <c r="E27" s="37"/>
+      <c r="F27" s="37"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="37"/>
+      <c r="I27" s="37"/>
+      <c r="J27" s="37"/>
+      <c r="K27" s="43"/>
     </row>
     <row r="28" spans="1:12" ht="25.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="28" t="s">
+      <c r="A28" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
-      <c r="I28" s="15"/>
-      <c r="J28" s="15"/>
-      <c r="K28" s="16"/>
+      <c r="B28" s="39"/>
+      <c r="C28" s="39"/>
+      <c r="D28" s="39"/>
+      <c r="E28" s="39"/>
+      <c r="F28" s="39"/>
+      <c r="G28" s="39"/>
+      <c r="H28" s="39"/>
+      <c r="I28" s="39"/>
+      <c r="J28" s="39"/>
+      <c r="K28" s="40"/>
     </row>
     <row r="29" spans="1:12" ht="25.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="29" t="s">
+      <c r="A29" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="B29" s="15"/>
-      <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="15"/>
-      <c r="F29" s="15"/>
-      <c r="G29" s="15"/>
-      <c r="H29" s="15"/>
-      <c r="I29" s="15"/>
-      <c r="J29" s="15"/>
-      <c r="K29" s="16"/>
+      <c r="B29" s="39"/>
+      <c r="C29" s="39"/>
+      <c r="D29" s="39"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="39"/>
+      <c r="I29" s="39"/>
+      <c r="J29" s="39"/>
+      <c r="K29" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1873,495 +1898,495 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
     </row>
     <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="39"/>
-      <c r="B3" s="39"/>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="39"/>
-      <c r="F3" s="39"/>
-      <c r="G3" s="40" t="s">
+      <c r="A3" s="27"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="H3" s="39"/>
+      <c r="H3" s="27"/>
     </row>
     <row r="4" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="39"/>
+      <c r="B4" s="27"/>
       <c r="C4" s="4"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
     </row>
     <row r="5" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="39"/>
-      <c r="B5" s="39"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
-      <c r="H5" s="39"/>
+      <c r="A5" s="27"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
     </row>
     <row r="6" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="39"/>
-      <c r="B6" s="41"/>
-      <c r="C6" s="39"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="39"/>
-      <c r="F6" s="39"/>
-      <c r="G6" s="39"/>
-      <c r="H6" s="39"/>
+      <c r="A6" s="27"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
     </row>
     <row r="7" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="39"/>
-      <c r="B7" s="41" t="s">
+      <c r="A7" s="27"/>
+      <c r="B7" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
-      <c r="G7" s="39"/>
-      <c r="H7" s="39"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
     </row>
     <row r="8" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="39"/>
-      <c r="B8" s="41" t="s">
+      <c r="A8" s="27"/>
+      <c r="B8" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="39"/>
-      <c r="H8" s="39"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
     </row>
     <row r="9" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="39"/>
-      <c r="B9" s="39"/>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
-      <c r="G9" s="39"/>
-      <c r="H9" s="39"/>
+      <c r="A9" s="27"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
     </row>
     <row r="10" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
-      <c r="H10" s="39"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
     </row>
     <row r="11" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
-      <c r="B11" s="39"/>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="39"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
     </row>
     <row r="12" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
-      <c r="B12" s="39"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="39"/>
-      <c r="H12" s="39"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
     </row>
     <row r="13" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="39"/>
-      <c r="B13" s="39"/>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="39"/>
-      <c r="H13" s="39"/>
+      <c r="A13" s="27"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
     </row>
     <row r="14" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="39"/>
-      <c r="C14" s="39"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="39"/>
-      <c r="H14" s="39"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
     </row>
     <row r="15" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
-      <c r="B15" s="39"/>
-      <c r="C15" s="39"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="39"/>
-      <c r="H15" s="39"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
     </row>
     <row r="16" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4"/>
-      <c r="B16" s="39"/>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="39"/>
-      <c r="H16" s="39"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
     </row>
     <row r="17" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="39"/>
-      <c r="B17" s="39"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="39"/>
-      <c r="H17" s="39"/>
+      <c r="A17" s="27"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
     </row>
     <row r="18" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="39"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="39"/>
+      <c r="B18" s="27"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
     </row>
     <row r="19" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
-      <c r="B19" s="39"/>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="39"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
     </row>
     <row r="20" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
-      <c r="B20" s="39"/>
-      <c r="C20" s="39"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="39"/>
-      <c r="G20" s="39"/>
-      <c r="H20" s="39"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
     </row>
     <row r="21" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="39"/>
-      <c r="B21" s="39"/>
-      <c r="C21" s="39"/>
-      <c r="D21" s="39"/>
-      <c r="E21" s="39"/>
-      <c r="F21" s="39"/>
-      <c r="G21" s="39"/>
-      <c r="H21" s="39"/>
+      <c r="A21" s="27"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
     </row>
     <row r="22" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="39"/>
-      <c r="C22" s="39"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="39"/>
-      <c r="H22" s="39"/>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
     </row>
     <row r="23" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
-      <c r="B23" s="39"/>
-      <c r="C23" s="39"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="39"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="39"/>
-      <c r="H23" s="39"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
     </row>
     <row r="24" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="39"/>
-      <c r="B24" s="39"/>
-      <c r="C24" s="39"/>
-      <c r="D24" s="39"/>
-      <c r="E24" s="39"/>
-      <c r="F24" s="39"/>
-      <c r="G24" s="39"/>
-      <c r="H24" s="39"/>
+      <c r="A24" s="27"/>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
     </row>
     <row r="25" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="39"/>
-      <c r="B25" s="39"/>
-      <c r="C25" s="39"/>
-      <c r="D25" s="39"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="39"/>
-      <c r="H25" s="39"/>
+      <c r="A25" s="27"/>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="27"/>
     </row>
     <row r="26" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B26" s="39"/>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="39"/>
-      <c r="G26" s="39"/>
-      <c r="H26" s="39"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="27"/>
+      <c r="H26" s="27"/>
     </row>
     <row r="27" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
-      <c r="B27" s="39"/>
-      <c r="C27" s="39"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="39"/>
-      <c r="F27" s="39"/>
-      <c r="G27" s="39"/>
-      <c r="H27" s="39"/>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="27"/>
     </row>
     <row r="28" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="39"/>
-      <c r="B28" s="39"/>
-      <c r="C28" s="39"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="39"/>
-      <c r="H28" s="39"/>
+      <c r="A28" s="27"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="27"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="27"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="27"/>
     </row>
     <row r="29" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="39"/>
-      <c r="B29" s="39"/>
-      <c r="C29" s="39"/>
-      <c r="D29" s="39"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="39"/>
+      <c r="A29" s="27"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="27"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="27"/>
     </row>
     <row r="30" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B30" s="39"/>
-      <c r="C30" s="39"/>
-      <c r="D30" s="39"/>
-      <c r="E30" s="39"/>
-      <c r="F30" s="39"/>
-      <c r="G30" s="39"/>
-      <c r="H30" s="39"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="27"/>
     </row>
     <row r="31" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
-      <c r="B31" s="39"/>
-      <c r="C31" s="39"/>
-      <c r="D31" s="39"/>
-      <c r="E31" s="39"/>
-      <c r="F31" s="39"/>
-      <c r="G31" s="39"/>
-      <c r="H31" s="39"/>
+      <c r="B31" s="27"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="27"/>
+      <c r="E31" s="27"/>
+      <c r="F31" s="27"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="27"/>
     </row>
     <row r="32" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="39"/>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="39"/>
-      <c r="E32" s="39"/>
-      <c r="F32" s="39"/>
-      <c r="G32" s="39"/>
-      <c r="H32" s="39"/>
+      <c r="A32" s="27"/>
+      <c r="B32" s="27"/>
+      <c r="C32" s="27"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="27"/>
+      <c r="G32" s="27"/>
+      <c r="H32" s="27"/>
     </row>
     <row r="33" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="39"/>
-      <c r="B33" s="39"/>
-      <c r="C33" s="39"/>
-      <c r="D33" s="39"/>
-      <c r="E33" s="39"/>
-      <c r="F33" s="39"/>
-      <c r="G33" s="39"/>
-      <c r="H33" s="39"/>
+      <c r="A33" s="27"/>
+      <c r="B33" s="27"/>
+      <c r="C33" s="27"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="27"/>
+      <c r="G33" s="27"/>
+      <c r="H33" s="27"/>
     </row>
     <row r="34" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B34" s="39"/>
-      <c r="C34" s="39"/>
-      <c r="D34" s="39"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="39"/>
-      <c r="G34" s="39"/>
-      <c r="H34" s="39"/>
+      <c r="B34" s="27"/>
+      <c r="C34" s="27"/>
+      <c r="D34" s="27"/>
+      <c r="E34" s="27"/>
+      <c r="F34" s="27"/>
+      <c r="G34" s="27"/>
+      <c r="H34" s="27"/>
     </row>
     <row r="35" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
-      <c r="B35" s="39"/>
-      <c r="C35" s="39"/>
-      <c r="D35" s="39"/>
-      <c r="E35" s="39"/>
-      <c r="F35" s="39"/>
-      <c r="G35" s="39"/>
-      <c r="H35" s="39"/>
+      <c r="B35" s="27"/>
+      <c r="C35" s="27"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="27"/>
+      <c r="H35" s="27"/>
     </row>
     <row r="36" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
-      <c r="B36" s="39"/>
-      <c r="C36" s="39"/>
-      <c r="D36" s="39"/>
-      <c r="E36" s="39"/>
-      <c r="F36" s="39"/>
-      <c r="G36" s="39"/>
-      <c r="H36" s="39"/>
+      <c r="B36" s="27"/>
+      <c r="C36" s="27"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="27"/>
+      <c r="F36" s="27"/>
+      <c r="G36" s="27"/>
+      <c r="H36" s="27"/>
     </row>
     <row r="37" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="39"/>
-      <c r="B37" s="39"/>
-      <c r="C37" s="39"/>
-      <c r="D37" s="39"/>
-      <c r="E37" s="39"/>
-      <c r="F37" s="39"/>
-      <c r="G37" s="39"/>
-      <c r="H37" s="39"/>
+      <c r="A37" s="27"/>
+      <c r="B37" s="27"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="27"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="27"/>
+      <c r="G37" s="27"/>
+      <c r="H37" s="27"/>
     </row>
     <row r="38" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B38" s="39"/>
-      <c r="C38" s="39"/>
-      <c r="D38" s="39"/>
-      <c r="E38" s="39"/>
-      <c r="F38" s="39"/>
-      <c r="G38" s="39"/>
-      <c r="H38" s="39"/>
+      <c r="B38" s="27"/>
+      <c r="C38" s="27"/>
+      <c r="D38" s="27"/>
+      <c r="E38" s="27"/>
+      <c r="F38" s="27"/>
+      <c r="G38" s="27"/>
+      <c r="H38" s="27"/>
     </row>
     <row r="39" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
-      <c r="B39" s="39"/>
-      <c r="C39" s="39"/>
-      <c r="D39" s="39"/>
-      <c r="E39" s="39"/>
-      <c r="F39" s="39"/>
-      <c r="G39" s="39"/>
-      <c r="H39" s="39"/>
+      <c r="B39" s="27"/>
+      <c r="C39" s="27"/>
+      <c r="D39" s="27"/>
+      <c r="E39" s="27"/>
+      <c r="F39" s="27"/>
+      <c r="G39" s="27"/>
+      <c r="H39" s="27"/>
     </row>
     <row r="40" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="39"/>
-      <c r="B40" s="39"/>
-      <c r="C40" s="39"/>
-      <c r="D40" s="39"/>
-      <c r="E40" s="39"/>
-      <c r="F40" s="39"/>
-      <c r="G40" s="39"/>
-      <c r="H40" s="39"/>
+      <c r="A40" s="27"/>
+      <c r="B40" s="27"/>
+      <c r="C40" s="27"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="27"/>
     </row>
     <row r="41" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="39"/>
-      <c r="B41" s="39"/>
-      <c r="C41" s="39"/>
-      <c r="D41" s="39"/>
-      <c r="E41" s="39"/>
-      <c r="F41" s="39"/>
-      <c r="G41" s="39"/>
-      <c r="H41" s="39"/>
+      <c r="A41" s="27"/>
+      <c r="B41" s="27"/>
+      <c r="C41" s="27"/>
+      <c r="D41" s="27"/>
+      <c r="E41" s="27"/>
+      <c r="F41" s="27"/>
+      <c r="G41" s="27"/>
+      <c r="H41" s="27"/>
     </row>
     <row r="42" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B42" s="39"/>
-      <c r="C42" s="39"/>
-      <c r="D42" s="39"/>
-      <c r="E42" s="39"/>
-      <c r="F42" s="39"/>
-      <c r="G42" s="39"/>
-      <c r="H42" s="39"/>
+      <c r="B42" s="27"/>
+      <c r="C42" s="27"/>
+      <c r="D42" s="27"/>
+      <c r="E42" s="27"/>
+      <c r="F42" s="27"/>
+      <c r="G42" s="27"/>
+      <c r="H42" s="27"/>
     </row>
     <row r="43" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="4"/>
-      <c r="B43" s="39"/>
-      <c r="C43" s="39"/>
-      <c r="D43" s="39"/>
-      <c r="E43" s="39"/>
-      <c r="F43" s="39"/>
-      <c r="G43" s="39"/>
-      <c r="H43" s="39"/>
+      <c r="B43" s="27"/>
+      <c r="C43" s="27"/>
+      <c r="D43" s="27"/>
+      <c r="E43" s="27"/>
+      <c r="F43" s="27"/>
+      <c r="G43" s="27"/>
+      <c r="H43" s="27"/>
     </row>
     <row r="44" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="39"/>
-      <c r="B44" s="39"/>
-      <c r="C44" s="39"/>
-      <c r="D44" s="39"/>
-      <c r="E44" s="39"/>
-      <c r="F44" s="39"/>
-      <c r="G44" s="39"/>
-      <c r="H44" s="39"/>
+      <c r="A44" s="27"/>
+      <c r="B44" s="27"/>
+      <c r="C44" s="27"/>
+      <c r="D44" s="27"/>
+      <c r="E44" s="27"/>
+      <c r="F44" s="27"/>
+      <c r="G44" s="27"/>
+      <c r="H44" s="27"/>
     </row>
     <row r="45" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="39"/>
-      <c r="B45" s="39"/>
-      <c r="C45" s="39"/>
-      <c r="D45" s="39"/>
-      <c r="E45" s="39"/>
-      <c r="F45" s="39"/>
-      <c r="G45" s="39"/>
-      <c r="H45" s="39"/>
+      <c r="A45" s="27"/>
+      <c r="B45" s="27"/>
+      <c r="C45" s="27"/>
+      <c r="D45" s="27"/>
+      <c r="E45" s="27"/>
+      <c r="F45" s="27"/>
+      <c r="G45" s="27"/>
+      <c r="H45" s="27"/>
     </row>
     <row r="46" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B46" s="39"/>
-      <c r="C46" s="39"/>
-      <c r="D46" s="39"/>
-      <c r="E46" s="39"/>
-      <c r="F46" s="39"/>
-      <c r="G46" s="39"/>
-      <c r="H46" s="39"/>
+      <c r="B46" s="27"/>
+      <c r="C46" s="27"/>
+      <c r="D46" s="27"/>
+      <c r="E46" s="27"/>
+      <c r="F46" s="27"/>
+      <c r="G46" s="27"/>
+      <c r="H46" s="27"/>
     </row>
     <row r="47" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A47" s="39"/>
-      <c r="B47" s="39"/>
-      <c r="C47" s="39"/>
-      <c r="D47" s="39"/>
-      <c r="E47" s="39"/>
-      <c r="F47" s="39"/>
-      <c r="G47" s="39"/>
-      <c r="H47" s="39"/>
+      <c r="A47" s="27"/>
+      <c r="B47" s="27"/>
+      <c r="C47" s="27"/>
+      <c r="D47" s="27"/>
+      <c r="E47" s="27"/>
+      <c r="F47" s="27"/>
+      <c r="G47" s="27"/>
+      <c r="H47" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>